<commit_message>
Outreach tracker: seed 23 real Bay Area contractors + scripts tab
Populate the Contractors tab with the named seed list from
CONTRACTOR_OUTREACH.md (SF/North Bay, East Bay, South Bay/Peninsula,
plus handyman breadth-fillers), all set to "Not contacted". Email and
phone are left blank on purpose — the outreach doc says verify each on
the company site / CSLB before contact — with the website and "where
found" captured in Notes so they're easy to verify.

Adds an "Outreach Scripts" tab (the offer, email template, IG DM, phone
opener, objection handling, consent/compliance rules, funnel target) so
the workbook is a self-contained outreach cockpit, not just a list.

Dropdowns, status color-coding, and the Pipeline Summary formulas carry
over and now count the 23 seeded rows.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/RenovateConnect_Outreach_Tracker.xlsx
+++ b/RenovateConnect_Outreach_Tracker.xlsx
@@ -10,7 +10,8 @@
     <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Contractors" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Homeowners" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Pipeline Summary" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Outreach Scripts" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Pipeline Summary" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Contractors'!$A$1:$P$1000</definedName>
@@ -26,7 +27,7 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -68,6 +69,16 @@
       <name val="Arial"/>
       <i val="1"/>
       <color rgb="00595959"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00333333"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -125,7 +136,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -153,6 +164,27 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -669,7 +701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P4"/>
+  <dimension ref="A1:P24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -773,240 +805,1168 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="inlineStr">
-        <is>
-          <t>Bright Kitchens LLC</t>
-        </is>
-      </c>
-      <c r="B2" s="5" t="inlineStr">
-        <is>
-          <t>Maria Lopez</t>
-        </is>
-      </c>
-      <c r="C2" s="5" t="inlineStr">
-        <is>
-          <t>maria@brightkitchens.example</t>
-        </is>
-      </c>
-      <c r="D2" s="5" t="inlineStr">
-        <is>
-          <t>(415) 555-0123</t>
-        </is>
-      </c>
-      <c r="E2" s="5" t="inlineStr">
+      <c r="A2" s="13" t="inlineStr">
+        <is>
+          <t>North Bay Construction</t>
+        </is>
+      </c>
+      <c r="B2" s="13" t="inlineStr"/>
+      <c r="C2" s="13" t="inlineStr"/>
+      <c r="D2" s="13" t="inlineStr"/>
+      <c r="E2" s="13" t="inlineStr">
+        <is>
+          <t>Whole home</t>
+        </is>
+      </c>
+      <c r="F2" s="13" t="inlineStr">
+        <is>
+          <t>Santa Rosa</t>
+        </is>
+      </c>
+      <c r="G2" s="13" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="H2" s="13" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="I2" s="13" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J2" s="14" t="inlineStr"/>
+      <c r="K2" s="14" t="inlineStr"/>
+      <c r="L2" s="14" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>GC, award-winning, established. Verify contact on site/CSLB.</t>
+        </is>
+      </c>
+      <c r="N2" s="13" t="inlineStr"/>
+      <c r="O2" s="13" t="inlineStr"/>
+      <c r="P2" s="13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="13" t="inlineStr">
+        <is>
+          <t>Inspired Builders Inc.</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr"/>
+      <c r="C3" s="13" t="inlineStr"/>
+      <c r="D3" s="13" t="inlineStr"/>
+      <c r="E3" s="13" t="inlineStr">
+        <is>
+          <t>Whole home</t>
+        </is>
+      </c>
+      <c r="F3" s="13" t="inlineStr">
+        <is>
+          <t>San Francisco</t>
+        </is>
+      </c>
+      <c r="G3" s="13" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="H3" s="13" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="I3" s="13" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J3" s="14" t="inlineStr"/>
+      <c r="K3" s="14" t="inlineStr"/>
+      <c r="L3" s="14" t="inlineStr"/>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>Design-build GC, strong customer-service reputation. Verify contact.</t>
+        </is>
+      </c>
+      <c r="N3" s="13" t="inlineStr"/>
+      <c r="O3" s="13" t="inlineStr"/>
+      <c r="P3" s="13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="13" t="inlineStr">
+        <is>
+          <t>Mayer's Construction &amp; Remodeling</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr"/>
+      <c r="C4" s="13" t="inlineStr"/>
+      <c r="D4" s="13" t="inlineStr"/>
+      <c r="E4" s="13" t="inlineStr">
+        <is>
+          <t>Whole home</t>
+        </is>
+      </c>
+      <c r="F4" s="13" t="inlineStr">
+        <is>
+          <t>San Francisco</t>
+        </is>
+      </c>
+      <c r="G4" s="13" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="H4" s="13" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="I4" s="13" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J4" s="14" t="inlineStr"/>
+      <c r="K4" s="14" t="inlineStr"/>
+      <c r="L4" s="14" t="inlineStr"/>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>Remodel GC, 40+ yrs. Verify contact.</t>
+        </is>
+      </c>
+      <c r="N4" s="13" t="n">
+        <v>40</v>
+      </c>
+      <c r="O4" s="13" t="inlineStr"/>
+      <c r="P4" s="13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>Bay Home Remodeling</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr"/>
+      <c r="C5" s="13" t="inlineStr"/>
+      <c r="D5" s="13" t="inlineStr"/>
+      <c r="E5" s="13" t="inlineStr">
+        <is>
+          <t>Whole home</t>
+        </is>
+      </c>
+      <c r="F5" s="13" t="inlineStr">
+        <is>
+          <t>San Francisco</t>
+        </is>
+      </c>
+      <c r="G5" s="13" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="H5" s="13" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="I5" s="13" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J5" s="13" t="inlineStr"/>
+      <c r="K5" s="13" t="inlineStr"/>
+      <c r="L5" s="13" t="inlineStr"/>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>Home remodeling, fast-growing, broad Bay coverage. Verify contact.</t>
+        </is>
+      </c>
+      <c r="N5" s="13" t="inlineStr"/>
+      <c r="O5" s="13" t="inlineStr"/>
+      <c r="P5" s="13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>Together Home Remodeling</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr"/>
+      <c r="C6" s="13" t="inlineStr"/>
+      <c r="D6" s="13" t="inlineStr"/>
+      <c r="E6" s="13" t="inlineStr">
+        <is>
+          <t>Whole home</t>
+        </is>
+      </c>
+      <c r="F6" s="13" t="inlineStr">
+        <is>
+          <t>San Francisco</t>
+        </is>
+      </c>
+      <c r="G6" s="13" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="H6" s="13" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="I6" s="13" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J6" s="13" t="inlineStr"/>
+      <c r="K6" s="13" t="inlineStr"/>
+      <c r="L6" s="13" t="inlineStr"/>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>GC, 5-star rated, serves whole Bay Area. Verify contact.</t>
+        </is>
+      </c>
+      <c r="N6" s="13" t="inlineStr"/>
+      <c r="O6" s="13" t="inlineStr"/>
+      <c r="P6" s="13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>Valex Construction</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr"/>
+      <c r="C7" s="13" t="inlineStr"/>
+      <c r="D7" s="13" t="inlineStr"/>
+      <c r="E7" s="13" t="inlineStr">
+        <is>
+          <t>Whole home</t>
+        </is>
+      </c>
+      <c r="F7" s="13" t="inlineStr">
+        <is>
+          <t>San Francisco</t>
+        </is>
+      </c>
+      <c r="G7" s="13" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="H7" s="13" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="I7" s="13" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J7" s="13" t="inlineStr"/>
+      <c r="K7" s="13" t="inlineStr"/>
+      <c r="L7" s="13" t="inlineStr"/>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>New build + remodel, 30+ yrs (Presler Konstantin). Verify contact.</t>
+        </is>
+      </c>
+      <c r="N7" s="13" t="n">
+        <v>30</v>
+      </c>
+      <c r="O7" s="13" t="inlineStr"/>
+      <c r="P7" s="13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t>Duffin Contractors</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr"/>
+      <c r="C8" s="13" t="inlineStr"/>
+      <c r="D8" s="13" t="inlineStr"/>
+      <c r="E8" s="13" t="inlineStr">
+        <is>
+          <t>Whole home</t>
+        </is>
+      </c>
+      <c r="F8" s="13" t="inlineStr">
+        <is>
+          <t>San Francisco</t>
+        </is>
+      </c>
+      <c r="G8" s="13" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="H8" s="13" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="I8" s="13" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J8" s="13" t="inlineStr"/>
+      <c r="K8" s="13" t="inlineStr"/>
+      <c r="L8" s="13" t="inlineStr"/>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>High-end custom GC, custom builds/additions. Verify contact.</t>
+        </is>
+      </c>
+      <c r="N8" s="13" t="inlineStr"/>
+      <c r="O8" s="13" t="inlineStr"/>
+      <c r="P8" s="13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>HDR Remodeling</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="inlineStr"/>
+      <c r="C9" s="13" t="inlineStr"/>
+      <c r="D9" s="13" t="inlineStr"/>
+      <c r="E9" s="13" t="inlineStr">
+        <is>
+          <t>Whole home</t>
+        </is>
+      </c>
+      <c r="F9" s="13" t="inlineStr">
+        <is>
+          <t>Berkeley</t>
+        </is>
+      </c>
+      <c r="G9" s="13" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="H9" s="13" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="I9" s="13" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J9" s="13" t="inlineStr"/>
+      <c r="K9" s="13" t="inlineStr"/>
+      <c r="L9" s="13" t="inlineStr"/>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>hdrremodeling.com. Design-build, since 1987, East Bay focus. Found via Houzz.</t>
+        </is>
+      </c>
+      <c r="N9" s="13" t="n">
+        <v>39</v>
+      </c>
+      <c r="O9" s="13" t="inlineStr"/>
+      <c r="P9" s="13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t>Custom Kitchens</t>
+        </is>
+      </c>
+      <c r="B10" s="13" t="inlineStr"/>
+      <c r="C10" s="13" t="inlineStr"/>
+      <c r="D10" s="13" t="inlineStr"/>
+      <c r="E10" s="13" t="inlineStr">
         <is>
           <t>Kitchen</t>
         </is>
       </c>
-      <c r="F2" s="5" t="inlineStr">
+      <c r="F10" s="13" t="inlineStr">
         <is>
           <t>Oakland</t>
         </is>
       </c>
-      <c r="G2" s="5" t="inlineStr">
+      <c r="G10" s="13" t="inlineStr">
         <is>
           <t>CA</t>
         </is>
       </c>
-      <c r="H2" s="5" t="inlineStr">
-        <is>
-          <t>Yelp</t>
-        </is>
-      </c>
-      <c r="I2" s="5" t="inlineStr">
-        <is>
-          <t>Signed up</t>
-        </is>
-      </c>
-      <c r="J2" s="9" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="K2" s="9" t="inlineStr">
-        <is>
-          <t>2026-06-08</t>
-        </is>
-      </c>
-      <c r="L2" s="9" t="inlineStr">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="M2" s="5" t="inlineStr">
-        <is>
-          <t>(example — delete me) Solid Yelp 4.8 with 60+ reviews. Verified license.</t>
-        </is>
-      </c>
-      <c r="N2" s="5" t="n">
-        <v>12</v>
-      </c>
-      <c r="O2" s="5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="P2" s="5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>Northgate Remodels</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>James Chen</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>james@northgate.example</t>
-        </is>
-      </c>
-      <c r="D3" s="5" t="inlineStr">
-        <is>
-          <t>(510) 555-0188</t>
-        </is>
-      </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="H10" s="13" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="I10" s="13" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J10" s="13" t="inlineStr"/>
+      <c r="K10" s="13" t="inlineStr"/>
+      <c r="L10" s="13" t="inlineStr"/>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>Kitchen/bath/design, est. 1950, NARI award. Found via Oakland Magazine.</t>
+        </is>
+      </c>
+      <c r="N10" s="13" t="n">
+        <v>75</v>
+      </c>
+      <c r="O10" s="13" t="inlineStr"/>
+      <c r="P10" s="13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>DLR Custom Builders</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="inlineStr"/>
+      <c r="C11" s="13" t="inlineStr"/>
+      <c r="D11" s="13" t="inlineStr"/>
+      <c r="E11" s="13" t="inlineStr">
         <is>
           <t>Whole home</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="F11" s="13" t="inlineStr">
         <is>
           <t>Berkeley</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="G11" s="13" t="inlineStr">
         <is>
           <t>CA</t>
         </is>
       </c>
-      <c r="H3" s="5" t="inlineStr">
-        <is>
-          <t>Instagram</t>
-        </is>
-      </c>
-      <c r="I3" s="5" t="inlineStr">
-        <is>
-          <t>Demo scheduled</t>
-        </is>
-      </c>
-      <c r="J3" s="9" t="inlineStr">
-        <is>
-          <t>2026-06-04</t>
-        </is>
-      </c>
-      <c r="K3" s="9" t="inlineStr">
-        <is>
-          <t>2026-06-09</t>
-        </is>
-      </c>
-      <c r="L3" s="9" t="inlineStr">
-        <is>
-          <t>2026-06-12</t>
-        </is>
-      </c>
-      <c r="M3" s="5" t="inlineStr">
-        <is>
-          <t>(example — delete me) Big IG following, posts before/afters weekly.</t>
-        </is>
-      </c>
-      <c r="N3" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="O3" s="5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="P3" s="5" t="inlineStr">
+      <c r="H11" s="13" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="I11" s="13" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J11" s="13" t="inlineStr"/>
+      <c r="K11" s="13" t="inlineStr"/>
+      <c r="L11" s="13" t="inlineStr"/>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>Custom GC — Berkeley/Oakland/Piedmont, 39 yrs. Verify contact.</t>
+        </is>
+      </c>
+      <c r="N11" s="13" t="n">
+        <v>39</v>
+      </c>
+      <c r="O11" s="13" t="inlineStr"/>
+      <c r="P11" s="13" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>Tilework by Tom</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>Tom Becker</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>tom@tilework.example</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>(415) 555-0140</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="inlineStr">
-        <is>
-          <t>Bathroom</t>
-        </is>
-      </c>
-      <c r="F4" s="5" t="inlineStr">
-        <is>
-          <t>San Francisco</t>
-        </is>
-      </c>
-      <c r="G4" s="5" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>Element Home Remodeling</t>
+        </is>
+      </c>
+      <c r="B12" s="13" t="inlineStr"/>
+      <c r="C12" s="13" t="inlineStr"/>
+      <c r="D12" s="13" t="inlineStr"/>
+      <c r="E12" s="13" t="inlineStr">
+        <is>
+          <t>Whole home</t>
+        </is>
+      </c>
+      <c r="F12" s="13" t="inlineStr">
+        <is>
+          <t>Oakland</t>
+        </is>
+      </c>
+      <c r="G12" s="13" t="inlineStr">
         <is>
           <t>CA</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
-        <is>
-          <t>Referral</t>
-        </is>
-      </c>
-      <c r="I4" s="5" t="inlineStr">
-        <is>
-          <t>Contacted</t>
-        </is>
-      </c>
-      <c r="J4" s="9" t="inlineStr">
-        <is>
-          <t>2026-06-06</t>
-        </is>
-      </c>
-      <c r="K4" s="9" t="inlineStr">
-        <is>
-          <t>2026-06-06</t>
-        </is>
-      </c>
-      <c r="L4" s="9" t="inlineStr">
-        <is>
-          <t>2026-06-13</t>
-        </is>
-      </c>
-      <c r="M4" s="5" t="inlineStr">
-        <is>
-          <t>(example — delete me) Referred by Jamie. Specializes in custom tile.</t>
-        </is>
-      </c>
-      <c r="N4" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="O4" s="5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="P4" s="5" t="inlineStr">
+      <c r="H12" s="13" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="I12" s="13" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J12" s="13" t="inlineStr"/>
+      <c r="K12" s="13" t="inlineStr"/>
+      <c r="L12" s="13" t="inlineStr"/>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>elementhomeremodelingeastbay.com. Design-build, East Bay.</t>
+        </is>
+      </c>
+      <c r="N12" s="13" t="inlineStr"/>
+      <c r="O12" s="13" t="inlineStr"/>
+      <c r="P12" s="13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>Building Lab</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="inlineStr"/>
+      <c r="C13" s="13" t="inlineStr"/>
+      <c r="D13" s="13" t="inlineStr"/>
+      <c r="E13" s="13" t="inlineStr">
+        <is>
+          <t>Whole home</t>
+        </is>
+      </c>
+      <c r="F13" s="13" t="inlineStr">
+        <is>
+          <t>Oakland</t>
+        </is>
+      </c>
+      <c r="G13" s="13" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="H13" s="13" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="I13" s="13" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J13" s="13" t="inlineStr"/>
+      <c r="K13" s="13" t="inlineStr"/>
+      <c r="L13" s="13" t="inlineStr"/>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>Remodel, award-winning (REMMIES winner). Verify contact.</t>
+        </is>
+      </c>
+      <c r="N13" s="13" t="inlineStr"/>
+      <c r="O13" s="13" t="inlineStr"/>
+      <c r="P13" s="13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>FMS Projects, Inc.</t>
+        </is>
+      </c>
+      <c r="B14" s="13" t="inlineStr"/>
+      <c r="C14" s="13" t="inlineStr"/>
+      <c r="D14" s="13" t="inlineStr"/>
+      <c r="E14" s="13" t="inlineStr">
+        <is>
+          <t>Kitchen</t>
+        </is>
+      </c>
+      <c r="F14" s="13" t="inlineStr">
+        <is>
+          <t>Oakland</t>
+        </is>
+      </c>
+      <c r="G14" s="13" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="H14" s="13" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="I14" s="13" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J14" s="13" t="inlineStr"/>
+      <c r="K14" s="13" t="inlineStr"/>
+      <c r="L14" s="13" t="inlineStr"/>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>High-end kitchen/bath, since 1987. Verify contact.</t>
+        </is>
+      </c>
+      <c r="N14" s="13" t="n">
+        <v>39</v>
+      </c>
+      <c r="O14" s="13" t="inlineStr"/>
+      <c r="P14" s="13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="13" t="inlineStr">
+        <is>
+          <t>Sigura Construction, Inc.</t>
+        </is>
+      </c>
+      <c r="B15" s="13" t="inlineStr"/>
+      <c r="C15" s="13" t="inlineStr"/>
+      <c r="D15" s="13" t="inlineStr"/>
+      <c r="E15" s="13" t="inlineStr">
+        <is>
+          <t>Whole home</t>
+        </is>
+      </c>
+      <c r="F15" s="13" t="inlineStr">
+        <is>
+          <t>San Jose</t>
+        </is>
+      </c>
+      <c r="G15" s="13" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="H15" s="13" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="I15" s="13" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J15" s="13" t="inlineStr"/>
+      <c r="K15" s="13" t="inlineStr"/>
+      <c r="L15" s="13" t="inlineStr"/>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>siguraconstruction.com. Custom home builder.</t>
+        </is>
+      </c>
+      <c r="N15" s="13" t="inlineStr"/>
+      <c r="O15" s="13" t="inlineStr"/>
+      <c r="P15" s="13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="13" t="inlineStr">
+        <is>
+          <t>EBCON Corporation</t>
+        </is>
+      </c>
+      <c r="B16" s="13" t="inlineStr"/>
+      <c r="C16" s="13" t="inlineStr"/>
+      <c r="D16" s="13" t="inlineStr"/>
+      <c r="E16" s="13" t="inlineStr">
+        <is>
+          <t>Whole home</t>
+        </is>
+      </c>
+      <c r="F16" s="13" t="inlineStr">
+        <is>
+          <t>Palo Alto</t>
+        </is>
+      </c>
+      <c r="G16" s="13" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="H16" s="13" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="I16" s="13" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J16" s="13" t="inlineStr"/>
+      <c r="K16" s="13" t="inlineStr"/>
+      <c r="L16" s="13" t="inlineStr"/>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>Remodel GC, Peninsula, 20+ yrs. Verify contact.</t>
+        </is>
+      </c>
+      <c r="N16" s="13" t="n">
+        <v>20</v>
+      </c>
+      <c r="O16" s="13" t="inlineStr"/>
+      <c r="P16" s="13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="13" t="inlineStr">
+        <is>
+          <t>Green Planet Remodeling, Inc.</t>
+        </is>
+      </c>
+      <c r="B17" s="13" t="inlineStr"/>
+      <c r="C17" s="13" t="inlineStr"/>
+      <c r="D17" s="13" t="inlineStr"/>
+      <c r="E17" s="13" t="inlineStr">
+        <is>
+          <t>Whole home</t>
+        </is>
+      </c>
+      <c r="F17" s="13" t="inlineStr">
+        <is>
+          <t>San Jose</t>
+        </is>
+      </c>
+      <c r="G17" s="13" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="H17" s="13" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="I17" s="13" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J17" s="13" t="inlineStr"/>
+      <c r="K17" s="13" t="inlineStr"/>
+      <c r="L17" s="13" t="inlineStr"/>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>Eco remodeling, 5x Best of Houzz. Verify contact.</t>
+        </is>
+      </c>
+      <c r="N17" s="13" t="inlineStr"/>
+      <c r="O17" s="13" t="inlineStr"/>
+      <c r="P17" s="13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="13" t="inlineStr">
+        <is>
+          <t>Level Up Home Remodeling</t>
+        </is>
+      </c>
+      <c r="B18" s="13" t="inlineStr"/>
+      <c r="C18" s="13" t="inlineStr"/>
+      <c r="D18" s="13" t="inlineStr"/>
+      <c r="E18" s="13" t="inlineStr">
+        <is>
+          <t>Whole home</t>
+        </is>
+      </c>
+      <c r="F18" s="13" t="inlineStr">
+        <is>
+          <t>San Jose</t>
+        </is>
+      </c>
+      <c r="G18" s="13" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="H18" s="13" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="I18" s="13" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J18" s="13" t="inlineStr"/>
+      <c r="K18" s="13" t="inlineStr"/>
+      <c r="L18" s="13" t="inlineStr"/>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>Remodel, Silicon Valley since 2010. Verify contact.</t>
+        </is>
+      </c>
+      <c r="N18" s="13" t="n">
+        <v>16</v>
+      </c>
+      <c r="O18" s="13" t="inlineStr"/>
+      <c r="P18" s="13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="13" t="inlineStr">
+        <is>
+          <t>Valley Boutique Builders</t>
+        </is>
+      </c>
+      <c r="B19" s="13" t="inlineStr"/>
+      <c r="C19" s="13" t="inlineStr"/>
+      <c r="D19" s="13" t="inlineStr"/>
+      <c r="E19" s="13" t="inlineStr">
+        <is>
+          <t>Whole home</t>
+        </is>
+      </c>
+      <c r="F19" s="13" t="inlineStr">
+        <is>
+          <t>San Jose</t>
+        </is>
+      </c>
+      <c r="G19" s="13" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="H19" s="13" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="I19" s="13" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J19" s="13" t="inlineStr"/>
+      <c r="K19" s="13" t="inlineStr"/>
+      <c r="L19" s="13" t="inlineStr"/>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>valleyboutiquebuilders.com. GC, San Jose.</t>
+        </is>
+      </c>
+      <c r="N19" s="13" t="inlineStr"/>
+      <c r="O19" s="13" t="inlineStr"/>
+      <c r="P19" s="13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="13" t="inlineStr">
+        <is>
+          <t>JEB3 Construction</t>
+        </is>
+      </c>
+      <c r="B20" s="13" t="inlineStr"/>
+      <c r="C20" s="13" t="inlineStr"/>
+      <c r="D20" s="13" t="inlineStr"/>
+      <c r="E20" s="13" t="inlineStr">
+        <is>
+          <t>Whole home</t>
+        </is>
+      </c>
+      <c r="F20" s="13" t="inlineStr">
+        <is>
+          <t>San Jose</t>
+        </is>
+      </c>
+      <c r="G20" s="13" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="H20" s="13" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="I20" s="13" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J20" s="13" t="inlineStr"/>
+      <c r="K20" s="13" t="inlineStr"/>
+      <c r="L20" s="13" t="inlineStr"/>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>Luxury renovation, since 2003. Verify contact.</t>
+        </is>
+      </c>
+      <c r="N20" s="13" t="n">
+        <v>23</v>
+      </c>
+      <c r="O20" s="13" t="inlineStr"/>
+      <c r="P20" s="13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="13" t="inlineStr">
+        <is>
+          <t>Woodcliff Builders</t>
+        </is>
+      </c>
+      <c r="B21" s="13" t="inlineStr"/>
+      <c r="C21" s="13" t="inlineStr"/>
+      <c r="D21" s="13" t="inlineStr"/>
+      <c r="E21" s="13" t="inlineStr">
+        <is>
+          <t>Whole home</t>
+        </is>
+      </c>
+      <c r="F21" s="13" t="inlineStr">
+        <is>
+          <t>Palo Alto</t>
+        </is>
+      </c>
+      <c r="G21" s="13" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="H21" s="13" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="I21" s="13" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J21" s="13" t="inlineStr"/>
+      <c r="K21" s="13" t="inlineStr"/>
+      <c r="L21" s="13" t="inlineStr"/>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>GC, Palo Alto area. Found via BuildZoom/Houzz. Verify contact.</t>
+        </is>
+      </c>
+      <c r="N21" s="13" t="inlineStr"/>
+      <c r="O21" s="13" t="inlineStr"/>
+      <c r="P21" s="13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="13" t="inlineStr">
+        <is>
+          <t>Longshore Handyman</t>
+        </is>
+      </c>
+      <c r="B22" s="13" t="inlineStr"/>
+      <c r="C22" s="13" t="inlineStr"/>
+      <c r="D22" s="13" t="inlineStr"/>
+      <c r="E22" s="13" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="F22" s="13" t="inlineStr">
+        <is>
+          <t>Walnut Creek</t>
+        </is>
+      </c>
+      <c r="G22" s="13" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="H22" s="13" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="I22" s="13" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J22" s="13" t="inlineStr"/>
+      <c r="K22" s="13" t="inlineStr"/>
+      <c r="L22" s="13" t="inlineStr"/>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>Home repair — Contra Costa/Alameda/Marin/SF. Text/call. Verify contact.</t>
+        </is>
+      </c>
+      <c r="N22" s="13" t="inlineStr"/>
+      <c r="O22" s="13" t="inlineStr"/>
+      <c r="P22" s="13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="13" t="inlineStr">
+        <is>
+          <t>F&amp;G Handyman (Gabriel Tun)</t>
+        </is>
+      </c>
+      <c r="B23" s="13" t="inlineStr"/>
+      <c r="C23" s="13" t="inlineStr"/>
+      <c r="D23" s="13" t="inlineStr"/>
+      <c r="E23" s="13" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="F23" s="13" t="inlineStr">
+        <is>
+          <t>San Jose</t>
+        </is>
+      </c>
+      <c r="G23" s="13" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="H23" s="13" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="I23" s="13" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J23" s="13" t="inlineStr"/>
+      <c r="K23" s="13" t="inlineStr"/>
+      <c r="L23" s="13" t="inlineStr"/>
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t>Handyman + small remodel. Text/call. Verify contact.</t>
+        </is>
+      </c>
+      <c r="N23" s="13" t="inlineStr"/>
+      <c r="O23" s="13" t="inlineStr"/>
+      <c r="P23" s="13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="13" t="inlineStr">
+        <is>
+          <t>Mr. Fix Bay Area</t>
+        </is>
+      </c>
+      <c r="B24" s="13" t="inlineStr"/>
+      <c r="C24" s="13" t="inlineStr"/>
+      <c r="D24" s="13" t="inlineStr"/>
+      <c r="E24" s="13" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="F24" s="13" t="inlineStr">
+        <is>
+          <t>San Jose</t>
+        </is>
+      </c>
+      <c r="G24" s="13" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="H24" s="13" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="I24" s="13" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J24" s="13" t="inlineStr"/>
+      <c r="K24" s="13" t="inlineStr"/>
+      <c r="L24" s="13" t="inlineStr"/>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>Full handyman, San Jose area. Text/call. Verify contact.</t>
+        </is>
+      </c>
+      <c r="N24" s="13" t="inlineStr"/>
+      <c r="O24" s="13" t="inlineStr"/>
+      <c r="P24" s="13" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1447,6 +2407,261 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:A42"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="100" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="15" t="inlineStr">
+        <is>
+          <t>Outreach Scripts &amp; Playbook</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="16" t="inlineStr">
+        <is>
+          <t>Channel priority</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>(1) warm intro if any  →  (2) Instagram DM for IG-active remodelers  →  (3) personalized email  →  (4) phone call to the office. Solo operators: text/call. Aim for 30–50 contacts to land 10–15 founders.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="16" t="inlineStr">
+        <is>
+          <t>The offer — why they say yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Free FOUNDING CONTRACTOR listing, framed as scarcity + status:</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>•  Free verified profile with top search placement at launch (no lead fees, ever — our anti-Thumbtack differentiator).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>•  "Verified Pro" badge + a spot in the launch "Verified Pros" carousel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>•  We do the setup for them — import photos and reviews, write the profile. Zero effort on their end.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>•  Free AI estimate tool their own customers can use.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>•  First N founders locked in (e.g. "first 20 contractors in the East Bay").</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Ask in return: permission to list them, a few portfolio photos, and ideally a testimonial / willingness to take the first leads.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="16" t="inlineStr">
+        <is>
+          <t>Email template</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>Subject: Free founding spot for [Company] on a new Bay Area renovation app</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="18" t="inlineStr">
+        <is>
+          <t>Hi [Name],</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="18" t="inlineStr">
+        <is>
+          <t>I came across [Company]'s work on [Houzz/Yelp/IG] — the [kitchen/bath/project] photos are exactly the quality we want to feature.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="18" t="inlineStr">
+        <is>
+          <t>We're launching RenovateConnect, a Bay Area app that connects homeowners with vetted contractors. We're hand-picking a small group of founding contractors to feature for free at launch — top placement, a Verified Pro badge, and no lead fees. We'll set up your whole profile for you from your existing photos and reviews; it takes you zero time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="18" t="inlineStr">
+        <is>
+          <t>Could I get your OK to feature [Company], and a few project photos to include? Happy to send a mockup of how your profile would look first.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="18" t="inlineStr">
+        <is>
+          <t>[Your name] · RenovateConnect</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="16" t="inlineStr">
+        <is>
+          <t>Instagram DM (shorter)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="18" t="inlineStr">
+        <is>
+          <t>Hi! Love [Company]'s remodels 🔨 We're launching a Bay Area renovation app and hand-picking a few founding contractors to feature free at launch — top spot, verified badge, no lead fees, we build the profile for you. Mind if we feature you? Can send a mockup first.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="16" t="inlineStr">
+        <is>
+          <t>Phone script (opener)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="18" t="inlineStr">
+        <is>
+          <t>"Hi, is this [Name]? I run RenovateConnect, a new Bay Area renovation app. We're featuring a handful of top contractors for free at launch — no cost, no lead fees. I'd love your permission to feature [Company]; we handle all the setup. Can I email you a mockup of your profile?"</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="16" t="inlineStr">
+        <is>
+          <t>Objection handling</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>"Is this another Thumbtack?"  →  "Opposite — we never charge per lead. Founding listing is free, top placement; you only ever pay a small % if you close a job through the app."</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>"I'm too busy / not taking work."  →  "No setup effort on you — we build it. And you control your availability in the app; turn off leads anytime."</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>"What does it cost later?"  →  Be honest: free founding listing now; future revenue is the 8% deposit commission on jobs booked through the app.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="16" t="inlineStr">
+        <is>
+          <t>Consent &amp; compliance (do this right)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>•  Get explicit permission before any business appears in the app. A short written OK (email reply "yes, go ahead") is enough to start — keep a record.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>•  Don't scrape/repost Yelp/Houzz reviews or photos without rights. Ask the contractor to supply their own, or get written permission for specific ones. Reviews are re-earned in-app, not copied.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>•  Use real, accurate info — verify the CSLB license # is active. Don't imply endorsement they didn't give.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>•  Offer easy opt-out — "tell us anytime and we'll remove your profile."</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="16" t="inlineStr">
+        <is>
+          <t>Funnel target (dense single-metro launch, e.g. East Bay)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>Contact 40  →  15 say yes  →  10 fully set up with photos = a credible launch roster.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="19" t="inlineStr">
+        <is>
+          <t>Recommendation: pick ONE metro and saturate it before expanding.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>